<commit_message>
fix: a pivot field with custom subtotals no longer gets a default subtotal item (#550)
A field added in code starts with the automatic subtotal, and a field Excel saved with custom subtotals loads with it too, because Excel leaves defaultSubtotal out and it defaults to true. AddSubtotal and AddMissingSubtotalItems gave such a field an item for every function, Automatic included, so it had a default item next to its custom ones. Excel writes none, on any axis. The field now gets no default item while it has a custom subtotal, and gets it back when the last custom one is removed. Subtotals and the saved subtotal attributes are unchanged, so a load and save of Excel's file writes what Excel wrote. The two pivot style reference files lose the default item they had next to sum, max and min.
</commit_message>
<xml_diff>
--- a/XLibur.Tests/Resource/Other/PivotTable/Style/Set_pivot_field_subtotals_style.xlsx
+++ b/XLibur.Tests/Resource/Other/PivotTable/Style/Set_pivot_field_subtotals_style.xlsx
@@ -131,18 +131,16 @@
   <location ref="A1" firstHeaderRow="0" firstDataRow="0" firstDataCol="0"/>
   <pivotFields count="3">
     <pivotField name="Name" axis="axisRow" subtotalTop="0" showAll="0" sumSubtotal="1">
-      <items count="4">
+      <items count="3">
         <item x="0"/>
         <item x="1"/>
-        <item t="default"/>
         <item t="sum"/>
       </items>
     </pivotField>
     <pivotField name="Month" axis="axisRow" subtotalTop="0" showAll="0" maxSubtotal="1" minSubtotal="1">
-      <items count="5">
+      <items count="4">
         <item x="0"/>
         <item x="1"/>
-        <item t="default"/>
         <item t="max"/>
         <item t="min"/>
       </items>

</xml_diff>